<commit_message>
Acabamento: linha em branco extra entre artigos; cabecalho com numero por cliente_tipo
- acabamento.py: 2 paragrafos em branco entre artigos (antes 1)
- _common.py: cabecalho passa a incluir sufixo ' NN' com a posicao
  da encomenda entre as do mesmo cliente_tipo (ex: '042/26 FR 15')
- historico.py: helper numero_por_cliente_tipo, calculado on-the-fly
  em criar()/editar() (nao persistido em JSON)
</commit_message>
<xml_diff>
--- a/data/historico_encomendas.xlsx
+++ b/data/historico_encomendas.xlsx
@@ -119,7 +119,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -155,6 +155,9 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -528,7 +531,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G15"/>
+  <dimension ref="A1:G17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -550,7 +553,7 @@
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Exportado em 12/05/2026 às 23:55</t>
+          <t>Exportado em 14/06/2026 às 18:37</t>
         </is>
       </c>
     </row>
@@ -731,12 +734,12 @@
           <t>• ALÇA DT 12 S/QUADROS ECO  ×2  — vamos
 • ALIMENTADOR REVERSIVEL C/PARAFINA  ×8  — lets go
 • Ninho  ×100
-• Pranchetas  ×5
+• Pranchetas  ×10
 • teste  ×5  — notas test</t>
         </is>
       </c>
       <c r="G8" s="11" t="n">
-        <v>120</v>
+        <v>125</v>
       </c>
     </row>
     <row r="9" ht="32" customHeight="1">
@@ -958,21 +961,94 @@
         <v>705</v>
       </c>
     </row>
-    <row r="15" ht="20" customHeight="1">
-      <c r="A15" s="13" t="inlineStr">
-        <is>
-          <t>Total de encomendas: 10</t>
-        </is>
-      </c>
-      <c r="G15" s="14">
-        <f>SUM(G5:G14)</f>
+    <row r="15" ht="48" customHeight="1">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>0041</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>14/06/2026</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>18:02</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>Diogo</t>
+        </is>
+      </c>
+      <c r="E15" s="13" t="inlineStr">
+        <is>
+          <t>FR</t>
+        </is>
+      </c>
+      <c r="F15" s="5" t="inlineStr">
+        <is>
+          <t>• ALIMENTADOR REVERSIVEL C/PARAFINA  ×400  — rgerg
+• ALÇA DT 12 S/QUADROS ECO  ×100  — r4f
+• ggg  ×60  — gg</t>
+        </is>
+      </c>
+      <c r="G15" s="7" t="n">
+        <v>560</v>
+      </c>
+    </row>
+    <row r="16" ht="32" customHeight="1">
+      <c r="A16" s="8" t="inlineStr">
+        <is>
+          <t>0042</t>
+        </is>
+      </c>
+      <c r="B16" s="9" t="inlineStr">
+        <is>
+          <t>14/06/2026</t>
+        </is>
+      </c>
+      <c r="C16" s="8" t="inlineStr">
+        <is>
+          <t>18:31</t>
+        </is>
+      </c>
+      <c r="D16" s="9" t="inlineStr">
+        <is>
+          <t>diogo</t>
+        </is>
+      </c>
+      <c r="E16" s="12" t="inlineStr">
+        <is>
+          <t>FR</t>
+        </is>
+      </c>
+      <c r="F16" s="9" t="inlineStr">
+        <is>
+          <t>• ALIMENTADOR REVERSIVEL C/PARAFINA  ×400
+• ALÇA DT 12 S/QUADROS ECO  ×300  — yuiuoujoi</t>
+        </is>
+      </c>
+      <c r="G16" s="11" t="n">
+        <v>700</v>
+      </c>
+    </row>
+    <row r="17" ht="20" customHeight="1">
+      <c r="A17" s="14" t="inlineStr">
+        <is>
+          <t>Total de encomendas: 12</t>
+        </is>
+      </c>
+      <c r="G17" s="15">
+        <f>SUM(G5:G16)</f>
         <v/>
       </c>
     </row>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A15:F15"/>
+    <mergeCell ref="A17:F17"/>
     <mergeCell ref="A1:G1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>